<commit_message>
Scenario 4 complete (outbound tracking + SF logging) + flow exports
- S4-B: EventBridge (Connect Contact Event, EMAIL/COMPLETED) -> Lambda outbound-log
  mode -> Outgoing EmailMessage on the SF Case (full in+out thread); IAM dynamodb:Query.
- S4-A native reporting validated (incoming/outgoing metrics + contact search).
- flows.tf: console-authored flows (Email-Inbound-Routing, Email-Agent-Guide) tracked
  drift-safe (lifecycle ignore_changes=all, guarded); consolidates email-inbound-flow.tf.
  Inbound Lambda-error branch fixed -> Email-Case-Queue.
- flow_debug var; docs/08 S4 = Built; docs/09 updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/implementation-status.xlsx
+++ b/docs/implementation-status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sateesh/D-Drive/MyProjects/aws-poc/manual/email-demo/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012F05D5-2519-E748-A56D-C02F1C17A2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A11513E-81E7-244A-9ADF-691188D818AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="181">
   <si>
     <t>#</t>
   </si>
@@ -253,13 +253,7 @@
     <t>Success: select work without duplicate effort</t>
   </si>
   <si>
-    <t>Needs self-selection + S5 duplicate-work alerts.</t>
-  </si>
-  <si>
     <t>Success: supervisors keep governance</t>
-  </si>
-  <si>
-    <t>Supervisor + native controls; cherry-pick governance not built.</t>
   </si>
   <si>
     <t>S4 Outbound tracking</t>
@@ -767,16 +761,6 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -802,6 +786,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1428,7 +1422,7 @@
         <v>5</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -1469,23 +1463,19 @@
       <c r="C27" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D27" s="8" t="s">
-        <v>72</v>
-      </c>
+      <c r="D27" s="8"/>
     </row>
     <row r="28" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>59</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="11" t="s">
-        <v>74</v>
-      </c>
+      <c r="D28" s="11"/>
     </row>
     <row r="29" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
@@ -1495,86 +1485,86 @@
     </row>
     <row r="30" spans="1:4" ht="40" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="41" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1585,66 +1575,66 @@
     </row>
     <row r="37" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>5</v>
@@ -1653,112 +1643,112 @@
     </row>
     <row r="42" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="40" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C49" s="10" t="s">
         <v>5</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1769,84 +1759,84 @@
     </row>
     <row r="51" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>114</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="40" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C56" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1857,122 +1847,122 @@
     </row>
     <row r="58" spans="1:4" ht="40" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="40" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C64" s="3"/>
       <c r="D64" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C66" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1983,111 +1973,111 @@
     </row>
     <row r="68" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C68" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="D68" s="6" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D69" s="8" t="s">
         <v>144</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D70" s="8" t="s">
         <v>144</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Future"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"Partial"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2109,10 +2099,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2126,13 +2116,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2140,13 +2130,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="40" x14ac:dyDescent="0.25">
@@ -2154,13 +2144,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2168,13 +2158,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2182,13 +2172,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2196,13 +2186,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="40" x14ac:dyDescent="0.25">
@@ -2210,13 +2200,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2224,13 +2214,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="40" x14ac:dyDescent="0.25">
@@ -2238,13 +2228,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2252,13 +2242,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="41" thickBot="1" x14ac:dyDescent="0.3">
@@ -2266,18 +2256,18 @@
         <v>11</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
S5 duplicate-work alerts: proactive warning of other open cases in the screen-pop
- salesforce.related_open_cases: query other OPEN cases for the customer's
  Contact/Account (excl. current); flow-mode returns dupCount + dupWarning.
- connect_flow/build_response carries the alert; inbound flow sets dupWarning attr;
  Email-Agent-Guide Detail view shows it (AttributeBar) on accept.
- docs/08: S5 = Built (duplicate-work alerts done); Custom-View polish = TODO.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/implementation-status.xlsx
+++ b/docs/implementation-status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sateesh/D-Drive/MyProjects/aws-poc/manual/email-demo/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A11513E-81E7-244A-9ADF-691188D818AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E03762-A636-E74F-9375-BABA39ADAC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -761,6 +761,16 @@
   <dxfs count="4">
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -786,16 +796,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1677,7 +1677,7 @@
         <v>100</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>101</v>
@@ -1731,7 +1731,7 @@
         <v>108</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D48" s="8" t="s">
         <v>109</v>
@@ -2071,13 +2071,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Future"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"Partial"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2267,7 +2267,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Update implementation-status.xlsx status tracker
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/implementation-status.xlsx
+++ b/docs/implementation-status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sateesh/D-Drive/MyProjects/aws-poc/manual/email-demo/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E03762-A636-E74F-9375-BABA39ADAC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895A09C5-BD0B-9244-A24B-76ABC2DD894E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="181">
   <si>
     <t>#</t>
   </si>
@@ -385,15 +385,9 @@
     <t>Route by Account Ownership</t>
   </si>
   <si>
-    <t>Account linked; routing by account owner reuses the Lambda pattern - not built.</t>
-  </si>
-  <si>
     <t>Route by Customer/Product/Order/Case Type/Business Rules</t>
   </si>
   <si>
-    <t>Lambda can query any Salesforce field; currently keys on Case Owner.</t>
-  </si>
-  <si>
     <t>Success: multiple variables simultaneously</t>
   </si>
   <si>
@@ -578,6 +572,12 @@
   </si>
   <si>
     <t>Rides on the self-selection setup. (remove manual assignment from agent/owner profile)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account linked; routing by account owner reuses the Lambda pattern </t>
+  </si>
+  <si>
+    <t>Lambda can query any Salesforce field; currently keys on Case Owner and Priority.</t>
   </si>
 </sst>
 </file>
@@ -1422,7 +1422,7 @@
         <v>5</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -1779,10 +1779,10 @@
         <v>115</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>116</v>
+        <v>179</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="40" x14ac:dyDescent="0.25">
@@ -1790,11 +1790,13 @@
         <v>112</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C53" s="3"/>
+        <v>116</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>5</v>
+      </c>
       <c r="D53" s="8" t="s">
-        <v>118</v>
+        <v>180</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -1802,13 +1804,13 @@
         <v>112</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -1816,13 +1818,13 @@
         <v>112</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
@@ -1830,13 +1832,13 @@
         <v>112</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1847,122 +1849,122 @@
     </row>
     <row r="58" spans="1:4" ht="40" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="40" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C64" s="3"/>
       <c r="D64" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C66" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1973,100 +1975,100 @@
     </row>
     <row r="68" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>142</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="C68" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="D68" s="6" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D69" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D70" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -2099,10 +2101,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2116,13 +2118,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2130,13 +2132,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="40" x14ac:dyDescent="0.25">
@@ -2144,13 +2146,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2158,13 +2160,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2172,13 +2174,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2186,13 +2188,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="40" x14ac:dyDescent="0.25">
@@ -2200,13 +2202,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2214,13 +2216,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="40" x14ac:dyDescent="0.25">
@@ -2228,13 +2230,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -2242,13 +2244,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="41" thickBot="1" x14ac:dyDescent="0.3">
@@ -2256,13 +2258,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>